<commit_message>
finalized with the sensors and actuator schematics
</commit_message>
<xml_diff>
--- a/hardware/BOM/PCB components.xlsx
+++ b/hardware/BOM/PCB components.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="164011"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12650" tabRatio="533"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12650" tabRatio="533" firstSheet="3" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="PWR MGT" sheetId="1" r:id="rId1"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="975" uniqueCount="356">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="976" uniqueCount="359">
   <si>
     <t>Component</t>
   </si>
@@ -46,9 +46,6 @@
     <t>Notes</t>
   </si>
   <si>
-    <t>buck converter</t>
-  </si>
-  <si>
     <t>input connector</t>
   </si>
   <si>
@@ -64,18 +61,12 @@
     <t>D1</t>
   </si>
   <si>
-    <t>Inductor</t>
-  </si>
-  <si>
     <t>L1</t>
   </si>
   <si>
     <t>C2</t>
   </si>
   <si>
-    <t>220 uF</t>
-  </si>
-  <si>
     <t>3.3. Volatage Regulator</t>
   </si>
   <si>
@@ -85,9 +76,6 @@
     <t>C4</t>
   </si>
   <si>
-    <t>fuse</t>
-  </si>
-  <si>
     <t>F1</t>
   </si>
   <si>
@@ -112,9 +100,6 @@
     <t>C1 is a bulk capacitor. Consider an electrolyte capacitor for this scenario</t>
   </si>
   <si>
-    <t>68 uH</t>
-  </si>
-  <si>
     <t>convert 5V to 3.3V for the microcontroller. Package type AMS1117 SOT-89-3L - 3.3 S:SOT-89-3L [simulation, used the MCP1702T-33]</t>
   </si>
   <si>
@@ -316,21 +301,6 @@
     <t>C474952</t>
   </si>
   <si>
-    <t>Buck Switching Regulator IC Fixed 5V 1 Output 3A TO-263-5L</t>
-  </si>
-  <si>
-    <t>HANSCHIP semiconductor</t>
-  </si>
-  <si>
-    <t>LM2595S-5.0RG</t>
-  </si>
-  <si>
-    <t>LCSC [https://www.lcsc.com/product-detail/C5145315.html?s_z=n_LM2595]</t>
-  </si>
-  <si>
-    <t>C5145315</t>
-  </si>
-  <si>
     <t>MICROCHIP</t>
   </si>
   <si>
@@ -361,12 +331,6 @@
     <t>CONN-TH_P5.08_KF128-5.08-2P</t>
   </si>
   <si>
-    <t>TO-263-5_L10.2-W9.9-P1.70-LS14.4-TL</t>
-  </si>
-  <si>
-    <t>TO-263-5-5P_L10.2-W8.7-H4.5-LS14.4-P1.70</t>
-  </si>
-  <si>
     <t>USB-C (USB TYPE-C) Receptacle Connector 16 Position Surface Mount</t>
   </si>
   <si>
@@ -1091,6 +1055,51 @@
   </si>
   <si>
     <t xml:space="preserve">L </t>
+  </si>
+  <si>
+    <t>33 uH</t>
+  </si>
+  <si>
+    <t xml:space="preserve">470uF / 25V </t>
+  </si>
+  <si>
+    <t>330uF / 10V or 16V</t>
+  </si>
+  <si>
+    <t>Inductor*</t>
+  </si>
+  <si>
+    <t>electrolytic capacitor*</t>
+  </si>
+  <si>
+    <t>fuse*</t>
+  </si>
+  <si>
+    <t>buck converter*</t>
+  </si>
+  <si>
+    <t>150kHz Buck Fixed 5V 3A TO-220-5 Voltage Regulators - DC DC Switching Regulators RoHS</t>
+  </si>
+  <si>
+    <t>HGSEMI</t>
+  </si>
+  <si>
+    <t>LM2595T-5.0</t>
+  </si>
+  <si>
+    <t>LCSC [https://www.lcsc.com/product-detail/C316671.html?s_z=n_LM2595]</t>
+  </si>
+  <si>
+    <t>C316671</t>
+  </si>
+  <si>
+    <t>TO-220-5L_L10.2-W4.5-P1.71-L</t>
+  </si>
+  <si>
+    <t>connector (water level)</t>
+  </si>
+  <si>
+    <t>using 3 2P connectors to connect via the 6pin holes down</t>
   </si>
 </sst>
 </file>
@@ -1577,7 +1586,7 @@
   <cols>
     <col min="1" max="1" width="20.08984375" style="12" customWidth="1"/>
     <col min="2" max="2" width="7.6328125" style="9" customWidth="1"/>
-    <col min="3" max="3" width="7.90625" style="9" customWidth="1"/>
+    <col min="3" max="3" width="12.1796875" style="9" customWidth="1"/>
     <col min="4" max="4" width="12.7265625" style="9" customWidth="1"/>
     <col min="5" max="5" width="13.453125" style="9" customWidth="1"/>
     <col min="6" max="6" width="13.08984375" style="9" customWidth="1"/>
@@ -1595,13 +1604,13 @@
         <v>0</v>
       </c>
       <c r="B1" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="C1" s="8" t="s">
-        <v>11</v>
-      </c>
       <c r="D1" s="8" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
       <c r="E1" s="8" t="s">
         <v>1</v>
@@ -1610,16 +1619,16 @@
         <v>2</v>
       </c>
       <c r="G1" s="8" t="s">
-        <v>106</v>
+        <v>96</v>
       </c>
       <c r="H1" s="8" t="s">
         <v>3</v>
       </c>
       <c r="I1" s="8" t="s">
-        <v>107</v>
+        <v>97</v>
       </c>
       <c r="J1" s="8" t="s">
-        <v>94</v>
+        <v>89</v>
       </c>
       <c r="K1" s="8" t="s">
         <v>4</v>
@@ -1648,627 +1657,627 @@
     </row>
     <row r="3" spans="1:13" s="22" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>334</v>
+        <v>322</v>
       </c>
       <c r="C3" s="2"/>
       <c r="D3" s="2" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>90</v>
+        <v>85</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>91</v>
+        <v>86</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>110</v>
+        <v>100</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>111</v>
+        <v>101</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>111</v>
+        <v>101</v>
       </c>
       <c r="J3" s="2">
         <v>0.91</v>
       </c>
       <c r="K3" s="2" t="s">
-        <v>95</v>
+        <v>90</v>
       </c>
       <c r="L3" s="2" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
       <c r="M3" s="21" t="s">
-        <v>88</v>
+        <v>83</v>
       </c>
     </row>
     <row r="4" spans="1:13" s="22" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
-        <v>20</v>
+        <v>349</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>149</v>
+        <v>137</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>150</v>
+        <v>138</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>151</v>
+        <v>139</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>152</v>
+        <v>140</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>152</v>
+        <v>140</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>155</v>
+        <v>143</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>155</v>
+        <v>143</v>
       </c>
       <c r="J4" s="2">
         <v>0.4</v>
       </c>
       <c r="K4" s="2" t="s">
-        <v>154</v>
+        <v>142</v>
       </c>
       <c r="L4" s="2" t="s">
-        <v>153</v>
+        <v>141</v>
       </c>
       <c r="M4" s="21" t="s">
-        <v>89</v>
+        <v>84</v>
       </c>
     </row>
     <row r="5" spans="1:13" s="22" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>161</v>
+        <v>149</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>158</v>
+        <v>146</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>158</v>
+        <v>146</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>157</v>
+        <v>145</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>156</v>
+        <v>144</v>
       </c>
       <c r="I5" s="2"/>
       <c r="J5" s="2">
         <v>1.34</v>
       </c>
       <c r="K5" s="2" t="s">
-        <v>159</v>
+        <v>147</v>
       </c>
       <c r="L5" s="2" t="s">
-        <v>160</v>
+        <v>148</v>
       </c>
       <c r="M5" s="21" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
     </row>
     <row r="6" spans="1:13" s="22" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C6" s="2"/>
       <c r="D6" s="2" t="s">
-        <v>144</v>
+        <v>132</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>142</v>
+        <v>130</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>143</v>
+        <v>131</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>146</v>
+        <v>134</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>147</v>
+        <v>135</v>
       </c>
       <c r="I6" s="2" t="s">
-        <v>146</v>
+        <v>134</v>
       </c>
       <c r="J6" s="2">
         <v>0.44</v>
       </c>
       <c r="K6" s="2" t="s">
-        <v>148</v>
+        <v>136</v>
       </c>
       <c r="L6" s="2" t="s">
-        <v>145</v>
+        <v>133</v>
       </c>
       <c r="M6" s="21" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
     </row>
     <row r="8" spans="1:13" s="24" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A8" s="3" t="s">
-        <v>7</v>
+        <v>350</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>135</v>
+        <v>123</v>
       </c>
       <c r="C8" s="4"/>
       <c r="D8" s="4" t="s">
-        <v>97</v>
+        <v>351</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>98</v>
+        <v>352</v>
       </c>
       <c r="F8" s="4" t="s">
-        <v>99</v>
+        <v>353</v>
       </c>
       <c r="G8" s="4" t="s">
-        <v>99</v>
+        <v>353</v>
       </c>
       <c r="H8" s="4" t="s">
-        <v>112</v>
+        <v>356</v>
       </c>
       <c r="I8" s="4" t="s">
-        <v>113</v>
+        <v>355</v>
       </c>
       <c r="J8" s="4">
-        <v>0.64</v>
+        <v>0.67</v>
       </c>
       <c r="K8" s="4" t="s">
-        <v>100</v>
+        <v>354</v>
       </c>
       <c r="L8" s="4" t="s">
-        <v>101</v>
+        <v>355</v>
       </c>
       <c r="M8" s="23" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
     </row>
     <row r="9" spans="1:13" s="24" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A9" s="3" t="s">
-        <v>35</v>
+        <v>348</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>16</v>
+        <v>345</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>162</v>
+        <v>150</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>163</v>
+        <v>151</v>
       </c>
       <c r="F9" s="4" t="s">
-        <v>163</v>
+        <v>151</v>
       </c>
       <c r="G9" s="4" t="s">
-        <v>157</v>
+        <v>145</v>
       </c>
       <c r="H9" s="4" t="s">
-        <v>166</v>
+        <v>154</v>
       </c>
       <c r="I9" s="4" t="s">
-        <v>166</v>
+        <v>154</v>
       </c>
       <c r="J9" s="4">
         <v>0.49</v>
       </c>
       <c r="K9" s="4" t="s">
-        <v>164</v>
+        <v>152</v>
       </c>
       <c r="L9" s="4" t="s">
-        <v>165</v>
+        <v>153</v>
       </c>
       <c r="M9" s="23"/>
     </row>
     <row r="10" spans="1:13" s="24" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A10" s="3" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="C10" s="4"/>
       <c r="D10" s="4" t="s">
-        <v>144</v>
+        <v>132</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>142</v>
+        <v>130</v>
       </c>
       <c r="F10" s="4" t="s">
-        <v>143</v>
+        <v>131</v>
       </c>
       <c r="G10" s="4" t="s">
-        <v>146</v>
+        <v>134</v>
       </c>
       <c r="H10" s="4" t="s">
-        <v>147</v>
+        <v>135</v>
       </c>
       <c r="I10" s="4" t="s">
-        <v>146</v>
+        <v>134</v>
       </c>
       <c r="J10" s="4">
         <v>0.44</v>
       </c>
       <c r="K10" s="4" t="s">
-        <v>148</v>
+        <v>136</v>
       </c>
       <c r="L10" s="4" t="s">
-        <v>145</v>
+        <v>133</v>
       </c>
       <c r="M10" s="23"/>
     </row>
     <row r="11" spans="1:13" s="24" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A11" s="3" t="s">
-        <v>13</v>
+        <v>347</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>29</v>
+        <v>344</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>176</v>
+        <v>164</v>
       </c>
       <c r="E11" s="4" t="s">
-        <v>174</v>
+        <v>162</v>
       </c>
       <c r="F11" s="4" t="s">
-        <v>175</v>
+        <v>163</v>
       </c>
       <c r="G11" s="4" t="s">
-        <v>355</v>
+        <v>343</v>
       </c>
       <c r="H11" s="4" t="s">
-        <v>179</v>
+        <v>167</v>
       </c>
       <c r="I11" s="4" t="s">
-        <v>180</v>
+        <v>168</v>
       </c>
       <c r="J11" s="4">
         <v>0.88</v>
       </c>
       <c r="K11" s="4" t="s">
-        <v>177</v>
+        <v>165</v>
       </c>
       <c r="L11" s="4" t="s">
-        <v>178</v>
+        <v>166</v>
       </c>
       <c r="M11" s="23"/>
     </row>
     <row r="12" spans="1:13" s="24" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A12" s="3" t="s">
-        <v>35</v>
+        <v>348</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>44</v>
+        <v>346</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>167</v>
+        <v>155</v>
       </c>
       <c r="E12" s="4" t="s">
-        <v>168</v>
+        <v>156</v>
       </c>
       <c r="F12" s="4" t="s">
-        <v>169</v>
+        <v>157</v>
       </c>
       <c r="G12" s="4" t="s">
-        <v>157</v>
+        <v>145</v>
       </c>
       <c r="H12" s="4" t="s">
-        <v>172</v>
+        <v>160</v>
       </c>
       <c r="I12" s="4" t="s">
-        <v>173</v>
+        <v>161</v>
       </c>
       <c r="J12" s="4">
         <v>0.55000000000000004</v>
       </c>
       <c r="K12" s="4" t="s">
-        <v>171</v>
+        <v>159</v>
       </c>
       <c r="L12" s="4" t="s">
-        <v>170</v>
+        <v>158</v>
       </c>
       <c r="M12" s="23"/>
     </row>
     <row r="14" spans="1:13" s="26" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A14" s="6" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>306</v>
+        <v>294</v>
       </c>
       <c r="C14" s="7"/>
       <c r="D14" s="7" t="s">
-        <v>103</v>
+        <v>93</v>
       </c>
       <c r="E14" s="7" t="s">
-        <v>102</v>
+        <v>92</v>
       </c>
       <c r="F14" s="7" t="s">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="G14" s="7" t="s">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="H14" s="7" t="s">
-        <v>108</v>
+        <v>98</v>
       </c>
       <c r="I14" s="7" t="s">
-        <v>109</v>
+        <v>99</v>
       </c>
       <c r="J14" s="7">
         <v>0.51</v>
       </c>
       <c r="K14" s="7" t="s">
-        <v>104</v>
+        <v>94</v>
       </c>
       <c r="L14" s="7" t="s">
-        <v>105</v>
+        <v>95</v>
       </c>
       <c r="M14" s="25" t="s">
-        <v>30</v>
+        <v>25</v>
       </c>
     </row>
     <row r="15" spans="1:13" s="26" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A15" s="6" t="s">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="C15" s="7" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="D15" s="7" t="s">
-        <v>184</v>
+        <v>172</v>
       </c>
       <c r="E15" s="7" t="s">
-        <v>183</v>
+        <v>171</v>
       </c>
       <c r="F15" s="7" t="s">
-        <v>185</v>
+        <v>173</v>
       </c>
       <c r="G15" s="7" t="s">
-        <v>181</v>
+        <v>169</v>
       </c>
       <c r="H15" s="7" t="s">
-        <v>182</v>
+        <v>170</v>
       </c>
       <c r="I15" s="7"/>
       <c r="J15" s="7">
         <v>0.59</v>
       </c>
       <c r="K15" s="7" t="s">
-        <v>186</v>
+        <v>174</v>
       </c>
       <c r="L15" s="7" t="s">
-        <v>187</v>
+        <v>175</v>
       </c>
       <c r="M15" s="25"/>
     </row>
     <row r="16" spans="1:13" s="26" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A16" s="6" t="s">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="C16" s="7" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="D16" s="7" t="s">
-        <v>184</v>
+        <v>172</v>
       </c>
       <c r="E16" s="7" t="s">
-        <v>183</v>
+        <v>171</v>
       </c>
       <c r="F16" s="7" t="s">
-        <v>185</v>
+        <v>173</v>
       </c>
       <c r="G16" s="7" t="s">
-        <v>181</v>
+        <v>169</v>
       </c>
       <c r="H16" s="7" t="s">
-        <v>182</v>
+        <v>170</v>
       </c>
       <c r="I16" s="7"/>
       <c r="J16" s="7">
         <v>0.59</v>
       </c>
       <c r="K16" s="7" t="s">
-        <v>186</v>
+        <v>174</v>
       </c>
       <c r="L16" s="7" t="s">
-        <v>187</v>
+        <v>175</v>
       </c>
       <c r="M16" s="25"/>
     </row>
     <row r="19" spans="1:13" s="29" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A19" s="16" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="B19" s="10" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="C19" s="27" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="D19" s="10" t="s">
-        <v>210</v>
+        <v>198</v>
       </c>
       <c r="E19" s="27" t="s">
-        <v>204</v>
+        <v>192</v>
       </c>
       <c r="F19" s="10" t="s">
-        <v>206</v>
+        <v>194</v>
       </c>
       <c r="G19" s="10" t="s">
-        <v>207</v>
+        <v>195</v>
       </c>
       <c r="H19" s="10" t="s">
-        <v>203</v>
+        <v>191</v>
       </c>
       <c r="I19" s="10"/>
       <c r="J19" s="10">
         <v>0.1</v>
       </c>
       <c r="K19" s="10" t="s">
-        <v>208</v>
+        <v>196</v>
       </c>
       <c r="L19" s="10" t="s">
-        <v>209</v>
+        <v>197</v>
       </c>
       <c r="M19" s="28"/>
     </row>
     <row r="20" spans="1:13" s="29" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A20" s="16" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="B20" s="10" t="s">
-        <v>85</v>
+        <v>80</v>
       </c>
       <c r="C20" s="27"/>
       <c r="D20" s="10" t="s">
-        <v>221</v>
+        <v>209</v>
       </c>
       <c r="E20" s="27" t="s">
-        <v>219</v>
+        <v>207</v>
       </c>
       <c r="F20" s="10" t="s">
-        <v>220</v>
+        <v>208</v>
       </c>
       <c r="G20" s="10" t="s">
-        <v>224</v>
+        <v>212</v>
       </c>
       <c r="H20" s="10" t="s">
-        <v>225</v>
+        <v>213</v>
       </c>
       <c r="I20" s="10" t="s">
-        <v>225</v>
+        <v>213</v>
       </c>
       <c r="J20" s="10">
         <v>0.04</v>
       </c>
       <c r="K20" s="10" t="s">
-        <v>222</v>
+        <v>210</v>
       </c>
       <c r="L20" s="10" t="s">
-        <v>223</v>
+        <v>211</v>
       </c>
       <c r="M20" s="28" t="s">
-        <v>46</v>
+        <v>41</v>
       </c>
     </row>
     <row r="21" spans="1:13" s="29" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A21" s="16" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="B21" s="10" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="C21" s="27" t="s">
-        <v>61</v>
+        <v>56</v>
       </c>
       <c r="D21" s="10" t="s">
-        <v>211</v>
+        <v>199</v>
       </c>
       <c r="E21" s="27" t="s">
-        <v>204</v>
+        <v>192</v>
       </c>
       <c r="F21" s="10" t="s">
-        <v>206</v>
+        <v>194</v>
       </c>
       <c r="G21" s="10" t="s">
-        <v>207</v>
+        <v>195</v>
       </c>
       <c r="H21" s="10" t="s">
-        <v>203</v>
+        <v>191</v>
       </c>
       <c r="I21" s="10"/>
       <c r="J21" s="10">
         <v>0.1</v>
       </c>
       <c r="K21" s="10" t="s">
-        <v>208</v>
+        <v>196</v>
       </c>
       <c r="L21" s="10" t="s">
-        <v>209</v>
+        <v>197</v>
       </c>
       <c r="M21" s="28"/>
     </row>
     <row r="22" spans="1:13" s="29" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A22" s="16" t="s">
-        <v>226</v>
+        <v>214</v>
       </c>
       <c r="B22" s="10" t="s">
-        <v>86</v>
+        <v>81</v>
       </c>
       <c r="C22" s="10"/>
       <c r="D22" s="10" t="s">
-        <v>227</v>
+        <v>215</v>
       </c>
       <c r="E22" s="10" t="s">
-        <v>228</v>
+        <v>216</v>
       </c>
       <c r="F22" s="10" t="s">
-        <v>229</v>
+        <v>217</v>
       </c>
       <c r="G22" s="10" t="s">
-        <v>229</v>
+        <v>217</v>
       </c>
       <c r="H22" s="10" t="s">
-        <v>232</v>
+        <v>220</v>
       </c>
       <c r="I22" s="10" t="s">
-        <v>232</v>
+        <v>220</v>
       </c>
       <c r="J22" s="10">
         <v>1.36</v>
       </c>
       <c r="K22" s="10" t="s">
-        <v>230</v>
+        <v>218</v>
       </c>
       <c r="L22" s="10" t="s">
-        <v>231</v>
+        <v>219</v>
       </c>
       <c r="M22" s="28" t="s">
-        <v>233</v>
+        <v>221</v>
       </c>
     </row>
     <row r="25" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A25" s="12" t="s">
-        <v>305</v>
+        <v>293</v>
       </c>
       <c r="J25" s="9">
         <f>SUM(J3:J22)</f>
-        <v>9.379999999999999</v>
+        <v>9.4099999999999984</v>
       </c>
     </row>
   </sheetData>
@@ -2303,13 +2312,13 @@
         <v>0</v>
       </c>
       <c r="B1" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="C1" s="8" t="s">
-        <v>11</v>
-      </c>
       <c r="D1" s="8" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
       <c r="E1" s="8" t="s">
         <v>1</v>
@@ -2318,16 +2327,16 @@
         <v>2</v>
       </c>
       <c r="G1" s="8" t="s">
-        <v>106</v>
+        <v>96</v>
       </c>
       <c r="H1" s="8" t="s">
         <v>3</v>
       </c>
       <c r="I1" s="8" t="s">
-        <v>107</v>
+        <v>97</v>
       </c>
       <c r="J1" s="8" t="s">
-        <v>94</v>
+        <v>89</v>
       </c>
       <c r="K1" s="8" t="s">
         <v>4</v>
@@ -2356,38 +2365,38 @@
     </row>
     <row r="3" spans="1:13" s="33" customFormat="1" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="30" t="s">
-        <v>134</v>
+        <v>122</v>
       </c>
       <c r="B3" s="31" t="s">
-        <v>331</v>
+        <v>319</v>
       </c>
       <c r="C3" s="31"/>
       <c r="D3" s="31" t="s">
-        <v>136</v>
+        <v>124</v>
       </c>
       <c r="E3" s="31" t="s">
-        <v>137</v>
+        <v>125</v>
       </c>
       <c r="F3" s="31" t="s">
-        <v>138</v>
+        <v>126</v>
       </c>
       <c r="G3" s="31" t="s">
-        <v>140</v>
+        <v>128</v>
       </c>
       <c r="H3" s="31" t="s">
-        <v>141</v>
+        <v>129</v>
       </c>
       <c r="I3" s="31" t="s">
-        <v>141</v>
+        <v>129</v>
       </c>
       <c r="J3" s="31">
         <v>5.61</v>
       </c>
       <c r="K3" s="31" t="s">
-        <v>195</v>
+        <v>183</v>
       </c>
       <c r="L3" s="31" t="s">
-        <v>139</v>
+        <v>127</v>
       </c>
       <c r="M3" s="32"/>
     </row>
@@ -2399,499 +2408,499 @@
     </row>
     <row r="5" spans="1:13" s="24" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A5" s="3" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>197</v>
+        <v>185</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>196</v>
+        <v>184</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>198</v>
+        <v>186</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>157</v>
+        <v>145</v>
       </c>
       <c r="H5" s="4" t="s">
-        <v>201</v>
+        <v>189</v>
       </c>
       <c r="I5" s="4" t="s">
-        <v>202</v>
+        <v>190</v>
       </c>
       <c r="J5" s="4">
         <v>0.42</v>
       </c>
       <c r="K5" s="4" t="s">
-        <v>200</v>
+        <v>188</v>
       </c>
       <c r="L5" s="4" t="s">
-        <v>199</v>
+        <v>187</v>
       </c>
       <c r="M5" s="23" t="s">
-        <v>50</v>
+        <v>45</v>
       </c>
     </row>
     <row r="6" spans="1:13" s="24" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A6" s="3" t="s">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>189</v>
+        <v>177</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>188</v>
+        <v>176</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>190</v>
+        <v>178</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>191</v>
+        <v>179</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>181</v>
+        <v>169</v>
       </c>
       <c r="H6" s="4" t="s">
-        <v>192</v>
+        <v>180</v>
       </c>
       <c r="I6" s="4"/>
       <c r="J6" s="4">
         <v>0.64</v>
       </c>
       <c r="K6" s="4" t="s">
-        <v>193</v>
+        <v>181</v>
       </c>
       <c r="L6" s="4" t="s">
-        <v>194</v>
+        <v>182</v>
       </c>
       <c r="M6" s="23" t="s">
-        <v>50</v>
+        <v>45</v>
       </c>
     </row>
     <row r="9" spans="1:13" s="26" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A9" s="6" t="s">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>335</v>
+        <v>323</v>
       </c>
       <c r="C9" s="7"/>
       <c r="D9" s="7" t="s">
-        <v>114</v>
+        <v>102</v>
       </c>
       <c r="E9" s="7" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="F9" s="7" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="G9" s="7" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="H9" s="7" t="s">
-        <v>117</v>
+        <v>105</v>
       </c>
       <c r="I9" s="7" t="s">
-        <v>118</v>
+        <v>106</v>
       </c>
       <c r="J9" s="7">
         <v>0.89</v>
       </c>
       <c r="K9" s="7" t="s">
-        <v>116</v>
+        <v>104</v>
       </c>
       <c r="L9" s="7" t="s">
-        <v>115</v>
+        <v>103</v>
       </c>
       <c r="M9" s="25"/>
     </row>
     <row r="10" spans="1:13" s="26" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A10" s="6" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="C10" s="7"/>
       <c r="D10" s="7" t="s">
-        <v>144</v>
+        <v>132</v>
       </c>
       <c r="E10" s="7" t="s">
-        <v>142</v>
+        <v>130</v>
       </c>
       <c r="F10" s="7" t="s">
-        <v>143</v>
+        <v>131</v>
       </c>
       <c r="G10" s="7" t="s">
-        <v>146</v>
+        <v>134</v>
       </c>
       <c r="H10" s="7" t="s">
-        <v>147</v>
+        <v>135</v>
       </c>
       <c r="I10" s="7" t="s">
-        <v>146</v>
+        <v>134</v>
       </c>
       <c r="J10" s="7">
         <v>0.44</v>
       </c>
       <c r="K10" s="7" t="s">
-        <v>148</v>
+        <v>136</v>
       </c>
       <c r="L10" s="7" t="s">
-        <v>145</v>
+        <v>133</v>
       </c>
       <c r="M10" s="25"/>
     </row>
     <row r="11" spans="1:13" s="26" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A11" s="6" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>53</v>
+        <v>48</v>
       </c>
       <c r="D11" s="7" t="s">
-        <v>205</v>
+        <v>193</v>
       </c>
       <c r="E11" s="34" t="s">
-        <v>204</v>
+        <v>192</v>
       </c>
       <c r="F11" s="7" t="s">
-        <v>206</v>
+        <v>194</v>
       </c>
       <c r="G11" s="7" t="s">
-        <v>207</v>
+        <v>195</v>
       </c>
       <c r="H11" s="7" t="s">
-        <v>203</v>
+        <v>191</v>
       </c>
       <c r="I11" s="7"/>
       <c r="J11" s="7">
         <v>0.1</v>
       </c>
       <c r="K11" s="7" t="s">
-        <v>208</v>
+        <v>196</v>
       </c>
       <c r="L11" s="7" t="s">
-        <v>209</v>
+        <v>197</v>
       </c>
       <c r="M11" s="25" t="s">
-        <v>55</v>
+        <v>50</v>
       </c>
     </row>
     <row r="12" spans="1:13" s="26" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A12" s="6" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="D12" s="7" t="s">
-        <v>205</v>
+        <v>193</v>
       </c>
       <c r="E12" s="34" t="s">
-        <v>204</v>
+        <v>192</v>
       </c>
       <c r="F12" s="7" t="s">
-        <v>206</v>
+        <v>194</v>
       </c>
       <c r="G12" s="7" t="s">
-        <v>207</v>
+        <v>195</v>
       </c>
       <c r="H12" s="7" t="s">
-        <v>203</v>
+        <v>191</v>
       </c>
       <c r="I12" s="7"/>
       <c r="J12" s="7">
         <v>0.1</v>
       </c>
       <c r="K12" s="7" t="s">
-        <v>208</v>
+        <v>196</v>
       </c>
       <c r="L12" s="7" t="s">
-        <v>209</v>
+        <v>197</v>
       </c>
       <c r="M12" s="25" t="s">
-        <v>56</v>
+        <v>51</v>
       </c>
     </row>
     <row r="15" spans="1:13" s="29" customFormat="1" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="16" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="B15" s="10" t="s">
-        <v>332</v>
+        <v>320</v>
       </c>
       <c r="C15" s="10"/>
       <c r="D15" s="10" t="s">
-        <v>121</v>
+        <v>109</v>
       </c>
       <c r="E15" s="10" t="s">
-        <v>119</v>
+        <v>107</v>
       </c>
       <c r="F15" s="10" t="s">
-        <v>120</v>
+        <v>108</v>
       </c>
       <c r="G15" s="10" t="s">
-        <v>124</v>
+        <v>112</v>
       </c>
       <c r="H15" s="10" t="s">
-        <v>125</v>
+        <v>113</v>
       </c>
       <c r="I15" s="10" t="s">
-        <v>126</v>
+        <v>114</v>
       </c>
       <c r="J15" s="10">
         <v>0.53</v>
       </c>
       <c r="K15" s="10" t="s">
-        <v>122</v>
+        <v>110</v>
       </c>
       <c r="L15" s="10" t="s">
-        <v>123</v>
+        <v>111</v>
       </c>
       <c r="M15" s="28"/>
     </row>
     <row r="16" spans="1:13" s="29" customFormat="1" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" s="16" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="B16" s="10" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="C16" s="10" t="s">
-        <v>61</v>
+        <v>56</v>
       </c>
       <c r="D16" s="10" t="s">
-        <v>211</v>
+        <v>199</v>
       </c>
       <c r="E16" s="27" t="s">
-        <v>204</v>
+        <v>192</v>
       </c>
       <c r="F16" s="10" t="s">
-        <v>206</v>
+        <v>194</v>
       </c>
       <c r="G16" s="10" t="s">
-        <v>207</v>
+        <v>195</v>
       </c>
       <c r="H16" s="10" t="s">
-        <v>203</v>
+        <v>191</v>
       </c>
       <c r="I16" s="10"/>
       <c r="J16" s="10">
         <v>0.1</v>
       </c>
       <c r="K16" s="10" t="s">
-        <v>208</v>
+        <v>196</v>
       </c>
       <c r="L16" s="10" t="s">
-        <v>209</v>
+        <v>197</v>
       </c>
       <c r="M16" s="28"/>
     </row>
     <row r="17" spans="1:13" s="29" customFormat="1" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A17" s="16" t="s">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="B17" s="10" t="s">
-        <v>63</v>
+        <v>58</v>
       </c>
       <c r="C17" s="10" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="D17" s="10" t="s">
-        <v>184</v>
+        <v>172</v>
       </c>
       <c r="E17" s="10" t="s">
-        <v>183</v>
+        <v>171</v>
       </c>
       <c r="F17" s="10" t="s">
-        <v>185</v>
+        <v>173</v>
       </c>
       <c r="G17" s="10" t="s">
-        <v>181</v>
+        <v>169</v>
       </c>
       <c r="H17" s="10" t="s">
-        <v>182</v>
+        <v>170</v>
       </c>
       <c r="I17" s="10"/>
       <c r="J17" s="10">
         <v>0.59</v>
       </c>
       <c r="K17" s="10" t="s">
-        <v>186</v>
+        <v>174</v>
       </c>
       <c r="L17" s="10" t="s">
-        <v>187</v>
+        <v>175</v>
       </c>
       <c r="M17" s="28"/>
     </row>
     <row r="18" spans="1:13" ht="14.5" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="20" spans="1:13" s="20" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A20" s="17" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="B20" s="11" t="s">
-        <v>333</v>
+        <v>321</v>
       </c>
       <c r="C20" s="11"/>
       <c r="D20" s="11" t="s">
-        <v>121</v>
+        <v>109</v>
       </c>
       <c r="E20" s="11" t="s">
-        <v>119</v>
+        <v>107</v>
       </c>
       <c r="F20" s="11" t="s">
-        <v>120</v>
+        <v>108</v>
       </c>
       <c r="G20" s="11" t="s">
-        <v>124</v>
+        <v>112</v>
       </c>
       <c r="H20" s="11" t="s">
-        <v>125</v>
+        <v>113</v>
       </c>
       <c r="I20" s="11" t="s">
-        <v>126</v>
+        <v>114</v>
       </c>
       <c r="J20" s="11">
         <v>0.53</v>
       </c>
       <c r="K20" s="11" t="s">
-        <v>122</v>
+        <v>110</v>
       </c>
       <c r="L20" s="11" t="s">
-        <v>123</v>
+        <v>111</v>
       </c>
       <c r="M20" s="35"/>
     </row>
     <row r="21" spans="1:13" s="20" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A21" s="17" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="B21" s="11" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="C21" s="11" t="s">
-        <v>61</v>
+        <v>56</v>
       </c>
       <c r="D21" s="11" t="s">
-        <v>211</v>
+        <v>199</v>
       </c>
       <c r="E21" s="36" t="s">
-        <v>204</v>
+        <v>192</v>
       </c>
       <c r="F21" s="11" t="s">
-        <v>206</v>
+        <v>194</v>
       </c>
       <c r="G21" s="11" t="s">
-        <v>207</v>
+        <v>195</v>
       </c>
       <c r="H21" s="11" t="s">
-        <v>203</v>
+        <v>191</v>
       </c>
       <c r="I21" s="11"/>
       <c r="J21" s="11">
         <v>0.1</v>
       </c>
       <c r="K21" s="11" t="s">
-        <v>208</v>
+        <v>196</v>
       </c>
       <c r="L21" s="11" t="s">
-        <v>209</v>
+        <v>197</v>
       </c>
       <c r="M21" s="35"/>
     </row>
     <row r="23" spans="1:13" s="40" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A23" s="37" t="s">
-        <v>62</v>
+        <v>57</v>
       </c>
       <c r="B23" s="38" t="s">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="C23" s="38"/>
       <c r="D23" s="38" t="s">
-        <v>297</v>
+        <v>285</v>
       </c>
       <c r="E23" s="38" t="s">
-        <v>298</v>
+        <v>286</v>
       </c>
       <c r="F23" s="38" t="s">
-        <v>299</v>
+        <v>287</v>
       </c>
       <c r="G23" s="38" t="s">
-        <v>299</v>
+        <v>287</v>
       </c>
       <c r="H23" s="38" t="s">
-        <v>302</v>
+        <v>290</v>
       </c>
       <c r="I23" s="38" t="s">
-        <v>302</v>
+        <v>290</v>
       </c>
       <c r="J23" s="38">
         <v>0.1</v>
       </c>
       <c r="K23" s="38" t="s">
-        <v>300</v>
+        <v>288</v>
       </c>
       <c r="L23" s="38" t="s">
-        <v>301</v>
+        <v>289</v>
       </c>
       <c r="M23" s="39"/>
     </row>
     <row r="24" spans="1:13" s="40" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A24" s="37" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="B24" s="38" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="C24" s="38" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="D24" s="38" t="s">
-        <v>210</v>
+        <v>198</v>
       </c>
       <c r="E24" s="41" t="s">
-        <v>204</v>
+        <v>192</v>
       </c>
       <c r="F24" s="38" t="s">
-        <v>206</v>
+        <v>194</v>
       </c>
       <c r="G24" s="38" t="s">
-        <v>207</v>
+        <v>195</v>
       </c>
       <c r="H24" s="38" t="s">
-        <v>203</v>
+        <v>191</v>
       </c>
       <c r="I24" s="38"/>
       <c r="J24" s="38">
         <v>0.1</v>
       </c>
       <c r="K24" s="38" t="s">
-        <v>208</v>
+        <v>196</v>
       </c>
       <c r="L24" s="38" t="s">
-        <v>209</v>
+        <v>197</v>
       </c>
       <c r="M24" s="39"/>
     </row>
     <row r="28" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A28" s="12" t="s">
-        <v>305</v>
+        <v>293</v>
       </c>
       <c r="J28" s="9">
         <f>SUM(J3:J24)</f>
@@ -2930,13 +2939,13 @@
         <v>0</v>
       </c>
       <c r="B1" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="C1" s="8" t="s">
-        <v>11</v>
-      </c>
       <c r="D1" s="8" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
       <c r="E1" s="8" t="s">
         <v>1</v>
@@ -2945,16 +2954,16 @@
         <v>2</v>
       </c>
       <c r="G1" s="8" t="s">
-        <v>106</v>
+        <v>96</v>
       </c>
       <c r="H1" s="8" t="s">
         <v>3</v>
       </c>
       <c r="I1" s="8" t="s">
-        <v>107</v>
+        <v>97</v>
       </c>
       <c r="J1" s="8" t="s">
-        <v>94</v>
+        <v>89</v>
       </c>
       <c r="K1" s="8" t="s">
         <v>4</v>
@@ -2975,304 +2984,304 @@
     </row>
     <row r="3" spans="1:13" s="22" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="B3" s="31" t="s">
-        <v>351</v>
+        <v>339</v>
       </c>
       <c r="C3" s="31"/>
       <c r="D3" s="2" t="s">
-        <v>127</v>
+        <v>115</v>
       </c>
       <c r="E3" s="31" t="s">
-        <v>128</v>
+        <v>116</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>129</v>
+        <v>117</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>129</v>
+        <v>117</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>132</v>
+        <v>120</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>133</v>
+        <v>121</v>
       </c>
       <c r="J3" s="2">
         <v>1.51</v>
       </c>
       <c r="K3" s="2" t="s">
-        <v>130</v>
+        <v>118</v>
       </c>
       <c r="L3" s="2" t="s">
-        <v>131</v>
+        <v>119</v>
       </c>
       <c r="M3" s="21" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
     </row>
     <row r="4" spans="1:13" s="22" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="B4" s="31" t="s">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="C4" s="31"/>
       <c r="D4" s="2" t="s">
-        <v>214</v>
+        <v>202</v>
       </c>
       <c r="E4" s="31" t="s">
-        <v>212</v>
+        <v>200</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>213</v>
+        <v>201</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>218</v>
+        <v>206</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>215</v>
+        <v>203</v>
       </c>
       <c r="I4" s="2"/>
       <c r="J4" s="2">
         <v>0.05</v>
       </c>
       <c r="K4" s="2" t="s">
-        <v>216</v>
+        <v>204</v>
       </c>
       <c r="L4" s="2" t="s">
-        <v>217</v>
+        <v>205</v>
       </c>
       <c r="M4" s="21"/>
     </row>
     <row r="5" spans="1:13" s="22" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="B5" s="31" t="s">
-        <v>87</v>
+        <v>82</v>
       </c>
       <c r="C5" s="31"/>
       <c r="D5" s="2" t="s">
-        <v>221</v>
+        <v>209</v>
       </c>
       <c r="E5" s="31" t="s">
-        <v>219</v>
+        <v>207</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>220</v>
+        <v>208</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>224</v>
+        <v>212</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>225</v>
+        <v>213</v>
       </c>
       <c r="I5" s="2" t="s">
-        <v>225</v>
+        <v>213</v>
       </c>
       <c r="J5" s="2">
         <v>0.04</v>
       </c>
       <c r="K5" s="2" t="s">
-        <v>222</v>
+        <v>210</v>
       </c>
       <c r="L5" s="2" t="s">
-        <v>223</v>
+        <v>211</v>
       </c>
       <c r="M5" s="21" t="s">
-        <v>46</v>
+        <v>41</v>
       </c>
     </row>
     <row r="6" spans="1:13" s="22" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="B6" s="31" t="s">
-        <v>84</v>
+        <v>79</v>
       </c>
       <c r="C6" s="31" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>210</v>
+        <v>198</v>
       </c>
       <c r="E6" s="31" t="s">
-        <v>204</v>
+        <v>192</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>206</v>
+        <v>194</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>207</v>
+        <v>195</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>203</v>
+        <v>191</v>
       </c>
       <c r="I6" s="2"/>
       <c r="J6" s="2">
         <v>0.1</v>
       </c>
       <c r="K6" s="2" t="s">
-        <v>208</v>
+        <v>196</v>
       </c>
       <c r="L6" s="2" t="s">
-        <v>209</v>
+        <v>197</v>
       </c>
       <c r="M6" s="21"/>
     </row>
     <row r="7" spans="1:13" s="22" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="B7" s="31" t="s">
-        <v>64</v>
+        <v>59</v>
       </c>
       <c r="C7" s="31" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>167</v>
+        <v>155</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>168</v>
+        <v>156</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>169</v>
+        <v>157</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>157</v>
+        <v>145</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>172</v>
+        <v>160</v>
       </c>
       <c r="I7" s="2" t="s">
-        <v>173</v>
+        <v>161</v>
       </c>
       <c r="J7" s="2">
         <v>0.55000000000000004</v>
       </c>
       <c r="K7" s="2" t="s">
-        <v>171</v>
+        <v>159</v>
       </c>
       <c r="L7" s="2" t="s">
-        <v>170</v>
+        <v>158</v>
       </c>
       <c r="M7" s="21"/>
     </row>
     <row r="8" spans="1:13" s="22" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A8" s="1" t="s">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="B8" s="31" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="C8" s="31"/>
       <c r="D8" s="2" t="s">
-        <v>214</v>
+        <v>202</v>
       </c>
       <c r="E8" s="31" t="s">
-        <v>212</v>
+        <v>200</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>213</v>
+        <v>201</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>218</v>
+        <v>206</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>215</v>
+        <v>203</v>
       </c>
       <c r="I8" s="2"/>
       <c r="J8" s="2">
         <v>0.05</v>
       </c>
       <c r="K8" s="2" t="s">
-        <v>216</v>
+        <v>204</v>
       </c>
       <c r="L8" s="2" t="s">
-        <v>217</v>
+        <v>205</v>
       </c>
       <c r="M8" s="21" t="s">
-        <v>46</v>
+        <v>41</v>
       </c>
     </row>
     <row r="9" spans="1:13" s="22" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A9" s="1" t="s">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="B9" s="31" t="s">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="C9" s="31" t="s">
-        <v>47</v>
+        <v>42</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>188</v>
+        <v>176</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>190</v>
+        <v>178</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>191</v>
+        <v>179</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>181</v>
+        <v>169</v>
       </c>
       <c r="H9" s="2" t="s">
-        <v>192</v>
+        <v>180</v>
       </c>
       <c r="I9" s="2"/>
       <c r="J9" s="2">
         <v>0.64</v>
       </c>
       <c r="K9" s="2" t="s">
-        <v>193</v>
+        <v>181</v>
       </c>
       <c r="L9" s="2" t="s">
-        <v>194</v>
+        <v>182</v>
       </c>
       <c r="M9" s="21"/>
     </row>
     <row r="10" spans="1:13" s="22" customFormat="1" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="1" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="B10" s="31" t="s">
-        <v>336</v>
+        <v>324</v>
       </c>
       <c r="C10" s="31"/>
       <c r="D10" s="2" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="E10" s="31" t="s">
-        <v>90</v>
+        <v>85</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>91</v>
+        <v>86</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>110</v>
+        <v>100</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>111</v>
+        <v>101</v>
       </c>
       <c r="I10" s="2" t="s">
-        <v>111</v>
+        <v>101</v>
       </c>
       <c r="J10" s="2">
         <v>0.91</v>
       </c>
       <c r="K10" s="2" t="s">
-        <v>95</v>
+        <v>90</v>
       </c>
       <c r="L10" s="2" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
       <c r="M10" s="21" t="s">
-        <v>88</v>
+        <v>83</v>
       </c>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.35">
@@ -3282,611 +3291,611 @@
     </row>
     <row r="12" spans="1:13" s="24" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A12" s="3" t="s">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="B12" s="42" t="s">
-        <v>352</v>
+        <v>340</v>
       </c>
       <c r="C12" s="42"/>
       <c r="D12" s="4" t="s">
-        <v>127</v>
+        <v>115</v>
       </c>
       <c r="E12" s="42" t="s">
-        <v>128</v>
+        <v>116</v>
       </c>
       <c r="F12" s="4" t="s">
-        <v>129</v>
+        <v>117</v>
       </c>
       <c r="G12" s="4" t="s">
-        <v>129</v>
+        <v>117</v>
       </c>
       <c r="H12" s="4" t="s">
-        <v>132</v>
+        <v>120</v>
       </c>
       <c r="I12" s="4" t="s">
-        <v>133</v>
+        <v>121</v>
       </c>
       <c r="J12" s="4">
         <v>1.51</v>
       </c>
       <c r="K12" s="4" t="s">
-        <v>130</v>
+        <v>118</v>
       </c>
       <c r="L12" s="4" t="s">
-        <v>131</v>
+        <v>119</v>
       </c>
       <c r="M12" s="23" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
     </row>
     <row r="13" spans="1:13" s="24" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A13" s="3" t="s">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="B13" s="42" t="s">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="C13" s="42"/>
       <c r="D13" s="4" t="s">
-        <v>214</v>
+        <v>202</v>
       </c>
       <c r="E13" s="42" t="s">
-        <v>212</v>
+        <v>200</v>
       </c>
       <c r="F13" s="4" t="s">
-        <v>213</v>
+        <v>201</v>
       </c>
       <c r="G13" s="4" t="s">
-        <v>218</v>
+        <v>206</v>
       </c>
       <c r="H13" s="4" t="s">
-        <v>215</v>
+        <v>203</v>
       </c>
       <c r="I13" s="4"/>
       <c r="J13" s="4">
         <v>0.05</v>
       </c>
       <c r="K13" s="4" t="s">
-        <v>216</v>
+        <v>204</v>
       </c>
       <c r="L13" s="4" t="s">
-        <v>217</v>
+        <v>205</v>
       </c>
       <c r="M13" s="23"/>
     </row>
     <row r="14" spans="1:13" s="24" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A14" s="3" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="B14" s="42" t="s">
-        <v>329</v>
+        <v>317</v>
       </c>
       <c r="C14" s="42"/>
       <c r="D14" s="4" t="s">
-        <v>221</v>
+        <v>209</v>
       </c>
       <c r="E14" s="42" t="s">
-        <v>219</v>
+        <v>207</v>
       </c>
       <c r="F14" s="4" t="s">
-        <v>220</v>
+        <v>208</v>
       </c>
       <c r="G14" s="4" t="s">
-        <v>224</v>
+        <v>212</v>
       </c>
       <c r="H14" s="4" t="s">
-        <v>225</v>
+        <v>213</v>
       </c>
       <c r="I14" s="4" t="s">
-        <v>225</v>
+        <v>213</v>
       </c>
       <c r="J14" s="4">
         <v>0.04</v>
       </c>
       <c r="K14" s="4" t="s">
-        <v>222</v>
+        <v>210</v>
       </c>
       <c r="L14" s="4" t="s">
-        <v>223</v>
+        <v>211</v>
       </c>
       <c r="M14" s="23" t="s">
-        <v>46</v>
+        <v>41</v>
       </c>
     </row>
     <row r="15" spans="1:13" s="24" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A15" s="3" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="B15" s="42" t="s">
-        <v>312</v>
+        <v>300</v>
       </c>
       <c r="C15" s="42" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>210</v>
+        <v>198</v>
       </c>
       <c r="E15" s="42" t="s">
-        <v>204</v>
+        <v>192</v>
       </c>
       <c r="F15" s="4" t="s">
-        <v>206</v>
+        <v>194</v>
       </c>
       <c r="G15" s="4" t="s">
-        <v>207</v>
+        <v>195</v>
       </c>
       <c r="H15" s="4" t="s">
-        <v>203</v>
+        <v>191</v>
       </c>
       <c r="I15" s="4"/>
       <c r="J15" s="4">
         <v>0.1</v>
       </c>
       <c r="K15" s="4" t="s">
-        <v>208</v>
+        <v>196</v>
       </c>
       <c r="L15" s="4" t="s">
-        <v>209</v>
+        <v>197</v>
       </c>
       <c r="M15" s="23"/>
     </row>
     <row r="16" spans="1:13" s="24" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A16" s="3" t="s">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="B16" s="42" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
       <c r="C16" s="42" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>167</v>
+        <v>155</v>
       </c>
       <c r="E16" s="4" t="s">
-        <v>168</v>
+        <v>156</v>
       </c>
       <c r="F16" s="4" t="s">
-        <v>169</v>
+        <v>157</v>
       </c>
       <c r="G16" s="4" t="s">
-        <v>157</v>
+        <v>145</v>
       </c>
       <c r="H16" s="4" t="s">
-        <v>172</v>
+        <v>160</v>
       </c>
       <c r="I16" s="4" t="s">
-        <v>173</v>
+        <v>161</v>
       </c>
       <c r="J16" s="4">
         <v>0.55000000000000004</v>
       </c>
       <c r="K16" s="4" t="s">
-        <v>171</v>
+        <v>159</v>
       </c>
       <c r="L16" s="4" t="s">
-        <v>170</v>
+        <v>158</v>
       </c>
       <c r="M16" s="23"/>
     </row>
     <row r="17" spans="1:13" s="24" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A17" s="3" t="s">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="B17" s="42" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="C17" s="42"/>
       <c r="D17" s="4" t="s">
-        <v>214</v>
+        <v>202</v>
       </c>
       <c r="E17" s="42" t="s">
-        <v>212</v>
+        <v>200</v>
       </c>
       <c r="F17" s="4" t="s">
-        <v>213</v>
+        <v>201</v>
       </c>
       <c r="G17" s="4" t="s">
-        <v>218</v>
+        <v>206</v>
       </c>
       <c r="H17" s="4" t="s">
-        <v>215</v>
+        <v>203</v>
       </c>
       <c r="I17" s="4"/>
       <c r="J17" s="4">
         <v>0.05</v>
       </c>
       <c r="K17" s="4" t="s">
-        <v>216</v>
+        <v>204</v>
       </c>
       <c r="L17" s="4" t="s">
-        <v>217</v>
+        <v>205</v>
       </c>
       <c r="M17" s="23" t="s">
-        <v>46</v>
+        <v>41</v>
       </c>
     </row>
     <row r="18" spans="1:13" s="24" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A18" s="3" t="s">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="B18" s="42" t="s">
-        <v>67</v>
+        <v>62</v>
       </c>
       <c r="C18" s="42" t="s">
-        <v>47</v>
+        <v>42</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>188</v>
+        <v>176</v>
       </c>
       <c r="E18" s="4" t="s">
-        <v>190</v>
+        <v>178</v>
       </c>
       <c r="F18" s="4" t="s">
-        <v>191</v>
+        <v>179</v>
       </c>
       <c r="G18" s="4" t="s">
-        <v>181</v>
+        <v>169</v>
       </c>
       <c r="H18" s="4" t="s">
-        <v>192</v>
+        <v>180</v>
       </c>
       <c r="I18" s="4"/>
       <c r="J18" s="4">
         <v>0.64</v>
       </c>
       <c r="K18" s="4" t="s">
-        <v>193</v>
+        <v>181</v>
       </c>
       <c r="L18" s="4" t="s">
-        <v>194</v>
+        <v>182</v>
       </c>
       <c r="M18" s="23"/>
     </row>
     <row r="19" spans="1:13" s="24" customFormat="1" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A19" s="3" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="B19" s="42" t="s">
-        <v>337</v>
+        <v>325</v>
       </c>
       <c r="C19" s="42"/>
       <c r="D19" s="4" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="E19" s="42" t="s">
-        <v>90</v>
+        <v>85</v>
       </c>
       <c r="F19" s="4" t="s">
-        <v>91</v>
+        <v>86</v>
       </c>
       <c r="G19" s="4" t="s">
-        <v>110</v>
+        <v>100</v>
       </c>
       <c r="H19" s="4" t="s">
-        <v>111</v>
+        <v>101</v>
       </c>
       <c r="I19" s="4" t="s">
-        <v>111</v>
+        <v>101</v>
       </c>
       <c r="J19" s="4">
         <v>0.91</v>
       </c>
       <c r="K19" s="4" t="s">
-        <v>95</v>
+        <v>90</v>
       </c>
       <c r="L19" s="4" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
       <c r="M19" s="23" t="s">
-        <v>88</v>
+        <v>83</v>
       </c>
     </row>
     <row r="22" spans="1:13" s="26" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A22" s="6" t="s">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="B22" s="34" t="s">
-        <v>353</v>
+        <v>341</v>
       </c>
       <c r="C22" s="34"/>
       <c r="D22" s="7" t="s">
-        <v>127</v>
+        <v>115</v>
       </c>
       <c r="E22" s="34" t="s">
-        <v>128</v>
+        <v>116</v>
       </c>
       <c r="F22" s="7" t="s">
-        <v>129</v>
+        <v>117</v>
       </c>
       <c r="G22" s="7" t="s">
-        <v>129</v>
+        <v>117</v>
       </c>
       <c r="H22" s="7" t="s">
-        <v>132</v>
+        <v>120</v>
       </c>
       <c r="I22" s="7" t="s">
-        <v>133</v>
+        <v>121</v>
       </c>
       <c r="J22" s="7">
         <v>1.51</v>
       </c>
       <c r="K22" s="7" t="s">
-        <v>130</v>
+        <v>118</v>
       </c>
       <c r="L22" s="7" t="s">
-        <v>131</v>
+        <v>119</v>
       </c>
       <c r="M22" s="25" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
     </row>
     <row r="23" spans="1:13" s="26" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A23" s="6" t="s">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="B23" s="34" t="s">
-        <v>82</v>
+        <v>77</v>
       </c>
       <c r="C23" s="34"/>
       <c r="D23" s="7" t="s">
-        <v>214</v>
+        <v>202</v>
       </c>
       <c r="E23" s="34" t="s">
-        <v>212</v>
+        <v>200</v>
       </c>
       <c r="F23" s="7" t="s">
-        <v>213</v>
+        <v>201</v>
       </c>
       <c r="G23" s="7" t="s">
-        <v>218</v>
+        <v>206</v>
       </c>
       <c r="H23" s="7" t="s">
-        <v>215</v>
+        <v>203</v>
       </c>
       <c r="I23" s="7"/>
       <c r="J23" s="7">
         <v>0.05</v>
       </c>
       <c r="K23" s="7" t="s">
-        <v>216</v>
+        <v>204</v>
       </c>
       <c r="L23" s="7" t="s">
-        <v>217</v>
+        <v>205</v>
       </c>
       <c r="M23" s="25"/>
     </row>
     <row r="24" spans="1:13" s="26" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A24" s="6" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="B24" s="34" t="s">
-        <v>330</v>
+        <v>318</v>
       </c>
       <c r="C24" s="34"/>
       <c r="D24" s="7" t="s">
-        <v>221</v>
+        <v>209</v>
       </c>
       <c r="E24" s="34" t="s">
-        <v>219</v>
+        <v>207</v>
       </c>
       <c r="F24" s="7" t="s">
-        <v>220</v>
+        <v>208</v>
       </c>
       <c r="G24" s="7" t="s">
-        <v>224</v>
+        <v>212</v>
       </c>
       <c r="H24" s="7" t="s">
-        <v>225</v>
+        <v>213</v>
       </c>
       <c r="I24" s="7" t="s">
-        <v>225</v>
+        <v>213</v>
       </c>
       <c r="J24" s="7">
         <v>0.04</v>
       </c>
       <c r="K24" s="7" t="s">
-        <v>222</v>
+        <v>210</v>
       </c>
       <c r="L24" s="7" t="s">
-        <v>223</v>
+        <v>211</v>
       </c>
       <c r="M24" s="25" t="s">
-        <v>46</v>
+        <v>41</v>
       </c>
     </row>
     <row r="25" spans="1:13" s="26" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A25" s="6" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="B25" s="34" t="s">
-        <v>313</v>
+        <v>301</v>
       </c>
       <c r="C25" s="34" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="D25" s="7" t="s">
-        <v>210</v>
+        <v>198</v>
       </c>
       <c r="E25" s="34" t="s">
-        <v>204</v>
+        <v>192</v>
       </c>
       <c r="F25" s="7" t="s">
-        <v>206</v>
+        <v>194</v>
       </c>
       <c r="G25" s="7" t="s">
-        <v>207</v>
+        <v>195</v>
       </c>
       <c r="H25" s="7" t="s">
-        <v>203</v>
+        <v>191</v>
       </c>
       <c r="I25" s="7"/>
       <c r="J25" s="7">
         <v>0.1</v>
       </c>
       <c r="K25" s="7" t="s">
-        <v>208</v>
+        <v>196</v>
       </c>
       <c r="L25" s="7" t="s">
-        <v>209</v>
+        <v>197</v>
       </c>
       <c r="M25" s="25"/>
     </row>
     <row r="26" spans="1:13" s="26" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A26" s="6" t="s">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="B26" s="34" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="C26" s="34" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="D26" s="7" t="s">
-        <v>167</v>
+        <v>155</v>
       </c>
       <c r="E26" s="7" t="s">
-        <v>168</v>
+        <v>156</v>
       </c>
       <c r="F26" s="7" t="s">
-        <v>169</v>
+        <v>157</v>
       </c>
       <c r="G26" s="7" t="s">
-        <v>157</v>
+        <v>145</v>
       </c>
       <c r="H26" s="7" t="s">
-        <v>172</v>
+        <v>160</v>
       </c>
       <c r="I26" s="7" t="s">
-        <v>173</v>
+        <v>161</v>
       </c>
       <c r="J26" s="7">
         <v>0.55000000000000004</v>
       </c>
       <c r="K26" s="7" t="s">
-        <v>171</v>
+        <v>159</v>
       </c>
       <c r="L26" s="7" t="s">
-        <v>170</v>
+        <v>158</v>
       </c>
       <c r="M26" s="25"/>
     </row>
     <row r="27" spans="1:13" s="26" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A27" s="6" t="s">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="B27" s="34" t="s">
-        <v>354</v>
+        <v>342</v>
       </c>
       <c r="C27" s="34"/>
       <c r="D27" s="7" t="s">
-        <v>214</v>
+        <v>202</v>
       </c>
       <c r="E27" s="34" t="s">
-        <v>212</v>
+        <v>200</v>
       </c>
       <c r="F27" s="7" t="s">
-        <v>213</v>
+        <v>201</v>
       </c>
       <c r="G27" s="7" t="s">
-        <v>218</v>
+        <v>206</v>
       </c>
       <c r="H27" s="7" t="s">
-        <v>215</v>
+        <v>203</v>
       </c>
       <c r="I27" s="7"/>
       <c r="J27" s="7">
         <v>0.05</v>
       </c>
       <c r="K27" s="7" t="s">
-        <v>216</v>
+        <v>204</v>
       </c>
       <c r="L27" s="7" t="s">
-        <v>217</v>
+        <v>205</v>
       </c>
       <c r="M27" s="25" t="s">
-        <v>46</v>
+        <v>41</v>
       </c>
     </row>
     <row r="28" spans="1:13" s="26" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A28" s="6" t="s">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="B28" s="34" t="s">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="C28" s="34" t="s">
-        <v>47</v>
+        <v>42</v>
       </c>
       <c r="D28" s="7" t="s">
-        <v>188</v>
+        <v>176</v>
       </c>
       <c r="E28" s="7" t="s">
-        <v>190</v>
+        <v>178</v>
       </c>
       <c r="F28" s="7" t="s">
-        <v>191</v>
+        <v>179</v>
       </c>
       <c r="G28" s="7" t="s">
-        <v>181</v>
+        <v>169</v>
       </c>
       <c r="H28" s="7" t="s">
-        <v>192</v>
+        <v>180</v>
       </c>
       <c r="I28" s="7"/>
       <c r="J28" s="7">
         <v>0.64</v>
       </c>
       <c r="K28" s="7" t="s">
-        <v>193</v>
+        <v>181</v>
       </c>
       <c r="L28" s="7" t="s">
-        <v>194</v>
+        <v>182</v>
       </c>
       <c r="M28" s="25"/>
     </row>
     <row r="29" spans="1:13" s="26" customFormat="1" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A29" s="6" t="s">
-        <v>48</v>
+        <v>43</v>
       </c>
       <c r="B29" s="34" t="s">
-        <v>338</v>
+        <v>326</v>
       </c>
       <c r="C29" s="34"/>
       <c r="D29" s="7" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="E29" s="34" t="s">
-        <v>90</v>
+        <v>85</v>
       </c>
       <c r="F29" s="7" t="s">
-        <v>91</v>
+        <v>86</v>
       </c>
       <c r="G29" s="7" t="s">
-        <v>110</v>
+        <v>100</v>
       </c>
       <c r="H29" s="7" t="s">
-        <v>111</v>
+        <v>101</v>
       </c>
       <c r="I29" s="7" t="s">
-        <v>111</v>
+        <v>101</v>
       </c>
       <c r="J29" s="7">
         <v>0.91</v>
       </c>
       <c r="K29" s="7" t="s">
-        <v>95</v>
+        <v>90</v>
       </c>
       <c r="L29" s="7" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
       <c r="M29" s="25" t="s">
-        <v>88</v>
+        <v>83</v>
       </c>
     </row>
     <row r="33" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A33" s="12" t="s">
-        <v>305</v>
+        <v>293</v>
       </c>
       <c r="J33" s="9">
         <f>SUM(J3:J30)</f>
@@ -3921,13 +3930,13 @@
         <v>0</v>
       </c>
       <c r="B1" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="C1" s="8" t="s">
-        <v>11</v>
-      </c>
       <c r="D1" s="8" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
       <c r="E1" s="8" t="s">
         <v>1</v>
@@ -3936,16 +3945,16 @@
         <v>2</v>
       </c>
       <c r="G1" s="8" t="s">
-        <v>106</v>
+        <v>96</v>
       </c>
       <c r="H1" s="8" t="s">
         <v>3</v>
       </c>
       <c r="I1" s="8" t="s">
-        <v>107</v>
+        <v>97</v>
       </c>
       <c r="J1" s="8" t="s">
-        <v>94</v>
+        <v>89</v>
       </c>
       <c r="K1" s="8" t="s">
         <v>4</v>
@@ -3965,898 +3974,900 @@
     </row>
     <row r="3" spans="1:14" s="22" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
-        <v>235</v>
+        <v>223</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>339</v>
+        <v>327</v>
       </c>
       <c r="C3" s="2"/>
       <c r="D3" s="2" t="s">
-        <v>240</v>
+        <v>228</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>90</v>
+        <v>85</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>239</v>
+        <v>227</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>239</v>
+        <v>227</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>244</v>
+        <v>232</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>244</v>
+        <v>232</v>
       </c>
       <c r="J3" s="2">
         <v>0.2</v>
       </c>
       <c r="K3" s="2" t="s">
-        <v>241</v>
+        <v>229</v>
       </c>
       <c r="L3" s="2" t="s">
-        <v>242</v>
+        <v>230</v>
       </c>
       <c r="M3" s="21" t="s">
-        <v>243</v>
+        <v>231</v>
       </c>
     </row>
     <row r="4" spans="1:14" s="22" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>314</v>
+        <v>302</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>245</v>
+        <v>233</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>272</v>
+        <v>260</v>
       </c>
       <c r="E4" s="31" t="s">
-        <v>204</v>
+        <v>192</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>206</v>
+        <v>194</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>207</v>
+        <v>195</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>203</v>
+        <v>191</v>
       </c>
       <c r="I4" s="2"/>
       <c r="J4" s="2">
         <v>0.1</v>
       </c>
       <c r="K4" s="2" t="s">
-        <v>208</v>
+        <v>196</v>
       </c>
       <c r="L4" s="2" t="s">
-        <v>209</v>
+        <v>197</v>
       </c>
       <c r="M4" s="21"/>
     </row>
     <row r="5" spans="1:14" s="22" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>315</v>
+        <v>303</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>238</v>
+        <v>226</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>273</v>
+        <v>261</v>
       </c>
       <c r="E5" s="31" t="s">
-        <v>204</v>
+        <v>192</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>206</v>
+        <v>194</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>207</v>
+        <v>195</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>203</v>
+        <v>191</v>
       </c>
       <c r="I5" s="2"/>
       <c r="J5" s="2">
         <v>0.1</v>
       </c>
       <c r="K5" s="2" t="s">
-        <v>208</v>
+        <v>196</v>
       </c>
       <c r="L5" s="2" t="s">
-        <v>209</v>
+        <v>197</v>
       </c>
       <c r="M5" s="21"/>
     </row>
     <row r="6" spans="1:14" s="22" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
-        <v>236</v>
+        <v>224</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>307</v>
+        <v>295</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>237</v>
+        <v>225</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>189</v>
+        <v>177</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>188</v>
+        <v>176</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>190</v>
+        <v>178</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>191</v>
+        <v>179</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>181</v>
+        <v>169</v>
       </c>
       <c r="I6" s="2" t="s">
-        <v>192</v>
+        <v>180</v>
       </c>
       <c r="J6" s="2"/>
       <c r="K6" s="2">
         <v>0.64</v>
       </c>
       <c r="L6" s="2" t="s">
-        <v>193</v>
+        <v>181</v>
       </c>
       <c r="M6" s="21" t="s">
-        <v>194</v>
+        <v>182</v>
       </c>
       <c r="N6" s="22" t="s">
-        <v>50</v>
+        <v>45</v>
       </c>
     </row>
     <row r="8" spans="1:14" s="24" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A8" s="3" t="s">
-        <v>246</v>
+        <v>234</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>340</v>
+        <v>328</v>
       </c>
       <c r="C8" s="4"/>
       <c r="D8" s="4" t="s">
-        <v>240</v>
+        <v>228</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>90</v>
+        <v>85</v>
       </c>
       <c r="F8" s="4" t="s">
-        <v>239</v>
+        <v>227</v>
       </c>
       <c r="G8" s="4" t="s">
-        <v>239</v>
+        <v>227</v>
       </c>
       <c r="H8" s="4" t="s">
-        <v>244</v>
+        <v>232</v>
       </c>
       <c r="I8" s="4" t="s">
-        <v>244</v>
+        <v>232</v>
       </c>
       <c r="J8" s="4">
         <v>0.2</v>
       </c>
       <c r="K8" s="4" t="s">
-        <v>241</v>
+        <v>229</v>
       </c>
       <c r="L8" s="4" t="s">
-        <v>242</v>
+        <v>230</v>
       </c>
       <c r="M8" s="23" t="s">
-        <v>243</v>
+        <v>231</v>
       </c>
     </row>
     <row r="9" spans="1:14" s="24" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A9" s="3" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>316</v>
+        <v>304</v>
       </c>
       <c r="C9" s="43" t="s">
-        <v>245</v>
+        <v>233</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>272</v>
+        <v>260</v>
       </c>
       <c r="E9" s="42" t="s">
-        <v>204</v>
+        <v>192</v>
       </c>
       <c r="F9" s="4" t="s">
-        <v>206</v>
+        <v>194</v>
       </c>
       <c r="G9" s="4" t="s">
-        <v>207</v>
+        <v>195</v>
       </c>
       <c r="H9" s="4" t="s">
-        <v>203</v>
+        <v>191</v>
       </c>
       <c r="I9" s="4"/>
       <c r="J9" s="4">
         <v>0.1</v>
       </c>
       <c r="K9" s="4" t="s">
-        <v>208</v>
+        <v>196</v>
       </c>
       <c r="L9" s="4" t="s">
-        <v>209</v>
+        <v>197</v>
       </c>
       <c r="M9" s="23"/>
     </row>
     <row r="10" spans="1:14" s="24" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A10" s="3" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>317</v>
+        <v>305</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>238</v>
+        <v>226</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>273</v>
+        <v>261</v>
       </c>
       <c r="E10" s="42" t="s">
-        <v>204</v>
+        <v>192</v>
       </c>
       <c r="F10" s="4" t="s">
-        <v>206</v>
+        <v>194</v>
       </c>
       <c r="G10" s="4" t="s">
-        <v>207</v>
+        <v>195</v>
       </c>
       <c r="H10" s="4" t="s">
-        <v>203</v>
+        <v>191</v>
       </c>
       <c r="I10" s="4"/>
       <c r="J10" s="4">
         <v>0.1</v>
       </c>
       <c r="K10" s="4" t="s">
-        <v>208</v>
+        <v>196</v>
       </c>
       <c r="L10" s="4" t="s">
-        <v>209</v>
+        <v>197</v>
       </c>
       <c r="M10" s="23"/>
     </row>
     <row r="11" spans="1:14" s="24" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A11" s="3" t="s">
-        <v>236</v>
+        <v>224</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>308</v>
+        <v>296</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>237</v>
+        <v>225</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>189</v>
+        <v>177</v>
       </c>
       <c r="E11" s="4" t="s">
-        <v>188</v>
+        <v>176</v>
       </c>
       <c r="F11" s="4" t="s">
-        <v>190</v>
+        <v>178</v>
       </c>
       <c r="G11" s="4" t="s">
-        <v>191</v>
+        <v>179</v>
       </c>
       <c r="H11" s="4" t="s">
-        <v>181</v>
+        <v>169</v>
       </c>
       <c r="I11" s="4" t="s">
-        <v>192</v>
+        <v>180</v>
       </c>
       <c r="J11" s="4"/>
       <c r="K11" s="4">
         <v>0.64</v>
       </c>
       <c r="L11" s="4" t="s">
-        <v>193</v>
+        <v>181</v>
       </c>
       <c r="M11" s="23" t="s">
-        <v>194</v>
+        <v>182</v>
       </c>
       <c r="N11" s="24" t="s">
-        <v>50</v>
+        <v>45</v>
       </c>
     </row>
     <row r="13" spans="1:14" s="26" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A13" s="6" t="s">
-        <v>247</v>
+        <v>235</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>341</v>
+        <v>329</v>
       </c>
       <c r="C13" s="7"/>
       <c r="D13" s="7" t="s">
-        <v>240</v>
+        <v>228</v>
       </c>
       <c r="E13" s="7" t="s">
-        <v>90</v>
+        <v>85</v>
       </c>
       <c r="F13" s="7" t="s">
-        <v>239</v>
+        <v>227</v>
       </c>
       <c r="G13" s="7" t="s">
-        <v>239</v>
+        <v>227</v>
       </c>
       <c r="H13" s="7" t="s">
-        <v>244</v>
+        <v>232</v>
       </c>
       <c r="I13" s="7" t="s">
-        <v>244</v>
+        <v>232</v>
       </c>
       <c r="J13" s="7">
         <v>0.2</v>
       </c>
       <c r="K13" s="7" t="s">
-        <v>241</v>
+        <v>229</v>
       </c>
       <c r="L13" s="7" t="s">
-        <v>242</v>
+        <v>230</v>
       </c>
       <c r="M13" s="25" t="s">
-        <v>243</v>
+        <v>231</v>
       </c>
     </row>
     <row r="14" spans="1:14" s="26" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A14" s="6" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>318</v>
+        <v>306</v>
       </c>
       <c r="C14" s="44" t="s">
-        <v>245</v>
+        <v>233</v>
       </c>
       <c r="D14" s="7" t="s">
-        <v>272</v>
+        <v>260</v>
       </c>
       <c r="E14" s="34" t="s">
-        <v>204</v>
+        <v>192</v>
       </c>
       <c r="F14" s="7" t="s">
-        <v>206</v>
+        <v>194</v>
       </c>
       <c r="G14" s="7" t="s">
-        <v>207</v>
+        <v>195</v>
       </c>
       <c r="H14" s="7" t="s">
-        <v>203</v>
+        <v>191</v>
       </c>
       <c r="I14" s="7"/>
       <c r="J14" s="7">
         <v>0.1</v>
       </c>
       <c r="K14" s="7" t="s">
-        <v>208</v>
+        <v>196</v>
       </c>
       <c r="L14" s="7" t="s">
-        <v>209</v>
+        <v>197</v>
       </c>
       <c r="M14" s="25"/>
     </row>
     <row r="15" spans="1:14" s="26" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A15" s="6" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>319</v>
+        <v>307</v>
       </c>
       <c r="C15" s="7" t="s">
-        <v>238</v>
+        <v>226</v>
       </c>
       <c r="D15" s="7" t="s">
-        <v>273</v>
+        <v>261</v>
       </c>
       <c r="E15" s="34" t="s">
-        <v>204</v>
+        <v>192</v>
       </c>
       <c r="F15" s="7" t="s">
-        <v>206</v>
+        <v>194</v>
       </c>
       <c r="G15" s="7" t="s">
-        <v>207</v>
+        <v>195</v>
       </c>
       <c r="H15" s="7" t="s">
-        <v>203</v>
+        <v>191</v>
       </c>
       <c r="I15" s="7"/>
       <c r="J15" s="7">
         <v>0.1</v>
       </c>
       <c r="K15" s="7" t="s">
-        <v>208</v>
+        <v>196</v>
       </c>
       <c r="L15" s="7" t="s">
-        <v>209</v>
+        <v>197</v>
       </c>
       <c r="M15" s="25"/>
     </row>
     <row r="16" spans="1:14" ht="14.5" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="17" spans="1:14" s="29" customFormat="1" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A17" s="16" t="s">
-        <v>248</v>
+        <v>236</v>
       </c>
       <c r="B17" s="10" t="s">
-        <v>342</v>
+        <v>330</v>
       </c>
       <c r="C17" s="10"/>
       <c r="D17" s="10" t="s">
+        <v>228</v>
+      </c>
+      <c r="E17" s="10" t="s">
+        <v>85</v>
+      </c>
+      <c r="F17" s="10" t="s">
+        <v>227</v>
+      </c>
+      <c r="G17" s="45" t="s">
+        <v>239</v>
+      </c>
+      <c r="H17" s="10" t="s">
         <v>240</v>
       </c>
-      <c r="E17" s="10" t="s">
-        <v>90</v>
-      </c>
-      <c r="F17" s="10" t="s">
-        <v>239</v>
-      </c>
-      <c r="G17" s="45" t="s">
-        <v>251</v>
-      </c>
-      <c r="H17" s="10" t="s">
-        <v>252</v>
-      </c>
       <c r="I17" s="10" t="s">
-        <v>253</v>
+        <v>241</v>
       </c>
       <c r="J17" s="10">
         <v>0.4</v>
       </c>
       <c r="K17" s="10" t="s">
-        <v>241</v>
+        <v>229</v>
       </c>
       <c r="L17" s="10" t="s">
-        <v>250</v>
+        <v>238</v>
       </c>
       <c r="M17" s="28" t="s">
-        <v>249</v>
+        <v>237</v>
       </c>
     </row>
     <row r="18" spans="1:14" ht="14.5" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="19" spans="1:14" s="20" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A19" s="17" t="s">
-        <v>247</v>
+        <v>357</v>
       </c>
       <c r="B19" s="11" t="s">
-        <v>343</v>
+        <v>331</v>
       </c>
       <c r="C19" s="11"/>
       <c r="D19" s="11" t="s">
-        <v>254</v>
+        <v>242</v>
       </c>
       <c r="E19" s="11" t="s">
-        <v>90</v>
+        <v>85</v>
       </c>
       <c r="F19" s="11" t="s">
-        <v>255</v>
+        <v>243</v>
       </c>
       <c r="G19" s="11" t="s">
-        <v>255</v>
+        <v>243</v>
       </c>
       <c r="H19" s="11" t="s">
-        <v>259</v>
+        <v>247</v>
       </c>
       <c r="I19" s="11" t="s">
-        <v>259</v>
+        <v>247</v>
       </c>
       <c r="J19" s="11">
         <v>0.2</v>
       </c>
       <c r="K19" s="11" t="s">
-        <v>257</v>
+        <v>245</v>
       </c>
       <c r="L19" s="11" t="s">
-        <v>256</v>
+        <v>244</v>
       </c>
       <c r="M19" s="35" t="s">
-        <v>258</v>
+        <v>246</v>
       </c>
     </row>
     <row r="20" spans="1:14" s="20" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A20" s="17" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="B20" s="11" t="s">
-        <v>320</v>
+        <v>308</v>
       </c>
       <c r="C20" s="46" t="s">
-        <v>245</v>
+        <v>233</v>
       </c>
       <c r="D20" s="11" t="s">
-        <v>272</v>
+        <v>260</v>
       </c>
       <c r="E20" s="36" t="s">
-        <v>204</v>
+        <v>192</v>
       </c>
       <c r="F20" s="11" t="s">
-        <v>206</v>
+        <v>194</v>
       </c>
       <c r="G20" s="11" t="s">
-        <v>207</v>
+        <v>195</v>
       </c>
       <c r="H20" s="11" t="s">
-        <v>203</v>
+        <v>191</v>
       </c>
       <c r="I20" s="11"/>
       <c r="J20" s="11">
         <v>0.1</v>
       </c>
       <c r="K20" s="11" t="s">
-        <v>208</v>
+        <v>196</v>
       </c>
       <c r="L20" s="11" t="s">
-        <v>209</v>
+        <v>197</v>
       </c>
       <c r="M20" s="35"/>
     </row>
     <row r="21" spans="1:14" s="20" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A21" s="17" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="B21" s="11" t="s">
-        <v>321</v>
+        <v>309</v>
       </c>
       <c r="C21" s="11" t="s">
-        <v>238</v>
+        <v>226</v>
       </c>
       <c r="D21" s="11" t="s">
-        <v>273</v>
+        <v>261</v>
       </c>
       <c r="E21" s="36" t="s">
-        <v>204</v>
+        <v>192</v>
       </c>
       <c r="F21" s="11" t="s">
-        <v>206</v>
+        <v>194</v>
       </c>
       <c r="G21" s="11" t="s">
-        <v>207</v>
+        <v>195</v>
       </c>
       <c r="H21" s="11" t="s">
-        <v>203</v>
+        <v>191</v>
       </c>
       <c r="I21" s="11"/>
       <c r="J21" s="11">
         <v>0.1</v>
       </c>
       <c r="K21" s="11" t="s">
-        <v>208</v>
+        <v>196</v>
       </c>
       <c r="L21" s="11" t="s">
-        <v>209</v>
+        <v>197</v>
       </c>
       <c r="M21" s="35"/>
     </row>
     <row r="23" spans="1:14" s="40" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A23" s="37" t="s">
-        <v>234</v>
+        <v>222</v>
       </c>
       <c r="B23" s="38" t="s">
-        <v>344</v>
+        <v>332</v>
       </c>
       <c r="C23" s="38"/>
       <c r="D23" s="38" t="s">
-        <v>240</v>
+        <v>228</v>
       </c>
       <c r="E23" s="38" t="s">
-        <v>90</v>
+        <v>85</v>
       </c>
       <c r="F23" s="38" t="s">
-        <v>239</v>
+        <v>227</v>
       </c>
       <c r="G23" s="38" t="s">
-        <v>239</v>
+        <v>227</v>
       </c>
       <c r="H23" s="38" t="s">
-        <v>244</v>
+        <v>232</v>
       </c>
       <c r="I23" s="38" t="s">
-        <v>244</v>
+        <v>232</v>
       </c>
       <c r="J23" s="38">
         <v>0.2</v>
       </c>
       <c r="K23" s="38" t="s">
-        <v>241</v>
+        <v>229</v>
       </c>
       <c r="L23" s="38" t="s">
-        <v>242</v>
+        <v>230</v>
       </c>
       <c r="M23" s="39" t="s">
-        <v>243</v>
+        <v>231</v>
       </c>
     </row>
     <row r="24" spans="1:14" s="40" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A24" s="37" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="B24" s="38" t="s">
-        <v>322</v>
+        <v>310</v>
       </c>
       <c r="C24" s="47" t="s">
-        <v>245</v>
+        <v>233</v>
       </c>
       <c r="D24" s="38" t="s">
-        <v>272</v>
+        <v>260</v>
       </c>
       <c r="E24" s="41" t="s">
-        <v>204</v>
+        <v>192</v>
       </c>
       <c r="F24" s="38" t="s">
-        <v>206</v>
+        <v>194</v>
       </c>
       <c r="G24" s="38" t="s">
-        <v>207</v>
+        <v>195</v>
       </c>
       <c r="H24" s="38" t="s">
-        <v>203</v>
+        <v>191</v>
       </c>
       <c r="I24" s="38"/>
       <c r="J24" s="38">
         <v>0.1</v>
       </c>
       <c r="K24" s="38" t="s">
-        <v>208</v>
+        <v>196</v>
       </c>
       <c r="L24" s="38" t="s">
-        <v>209</v>
+        <v>197</v>
       </c>
       <c r="M24" s="39"/>
     </row>
     <row r="25" spans="1:14" s="40" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A25" s="37" t="s">
-        <v>236</v>
+        <v>224</v>
       </c>
       <c r="B25" s="38" t="s">
-        <v>309</v>
+        <v>297</v>
       </c>
       <c r="C25" s="38" t="s">
-        <v>237</v>
+        <v>225</v>
       </c>
       <c r="D25" s="38" t="s">
-        <v>189</v>
+        <v>177</v>
       </c>
       <c r="E25" s="38" t="s">
-        <v>188</v>
+        <v>176</v>
       </c>
       <c r="F25" s="38" t="s">
-        <v>190</v>
+        <v>178</v>
       </c>
       <c r="G25" s="38" t="s">
-        <v>191</v>
+        <v>179</v>
       </c>
       <c r="H25" s="38" t="s">
-        <v>181</v>
+        <v>169</v>
       </c>
       <c r="I25" s="38" t="s">
-        <v>192</v>
+        <v>180</v>
       </c>
       <c r="J25" s="38"/>
       <c r="K25" s="38">
         <v>0.64</v>
       </c>
       <c r="L25" s="38" t="s">
-        <v>193</v>
+        <v>181</v>
       </c>
       <c r="M25" s="39" t="s">
-        <v>194</v>
+        <v>182</v>
       </c>
       <c r="N25" s="40" t="s">
-        <v>50</v>
+        <v>45</v>
       </c>
     </row>
     <row r="27" spans="1:14" s="51" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A27" s="48" t="s">
-        <v>260</v>
+        <v>248</v>
       </c>
       <c r="B27" s="49" t="s">
-        <v>345</v>
+        <v>333</v>
       </c>
       <c r="C27" s="49"/>
       <c r="D27" s="49" t="s">
-        <v>240</v>
+        <v>228</v>
       </c>
       <c r="E27" s="49" t="s">
-        <v>90</v>
+        <v>85</v>
       </c>
       <c r="F27" s="49" t="s">
-        <v>239</v>
+        <v>227</v>
       </c>
       <c r="G27" s="49" t="s">
-        <v>239</v>
+        <v>227</v>
       </c>
       <c r="H27" s="49" t="s">
-        <v>244</v>
+        <v>232</v>
       </c>
       <c r="I27" s="49" t="s">
-        <v>244</v>
+        <v>232</v>
       </c>
       <c r="J27" s="49">
         <v>0.2</v>
       </c>
       <c r="K27" s="49" t="s">
-        <v>241</v>
+        <v>229</v>
       </c>
       <c r="L27" s="49" t="s">
-        <v>242</v>
+        <v>230</v>
       </c>
       <c r="M27" s="50" t="s">
-        <v>243</v>
+        <v>231</v>
       </c>
     </row>
     <row r="28" spans="1:14" s="51" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A28" s="48" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="B28" s="49" t="s">
-        <v>323</v>
+        <v>311</v>
       </c>
       <c r="C28" s="52" t="s">
-        <v>245</v>
+        <v>233</v>
       </c>
       <c r="D28" s="49" t="s">
-        <v>272</v>
+        <v>260</v>
       </c>
       <c r="E28" s="53" t="s">
-        <v>204</v>
+        <v>192</v>
       </c>
       <c r="F28" s="49" t="s">
-        <v>206</v>
+        <v>194</v>
       </c>
       <c r="G28" s="49" t="s">
-        <v>207</v>
+        <v>195</v>
       </c>
       <c r="H28" s="49" t="s">
-        <v>203</v>
+        <v>191</v>
       </c>
       <c r="I28" s="49"/>
       <c r="J28" s="49">
         <v>0.1</v>
       </c>
       <c r="K28" s="49" t="s">
-        <v>208</v>
+        <v>196</v>
       </c>
       <c r="L28" s="49" t="s">
-        <v>209</v>
+        <v>197</v>
       </c>
       <c r="M28" s="50"/>
     </row>
     <row r="29" spans="1:14" s="51" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A29" s="48" t="s">
-        <v>236</v>
+        <v>224</v>
       </c>
       <c r="B29" s="49" t="s">
-        <v>310</v>
+        <v>298</v>
       </c>
       <c r="C29" s="49" t="s">
-        <v>237</v>
+        <v>225</v>
       </c>
       <c r="D29" s="49" t="s">
-        <v>189</v>
+        <v>177</v>
       </c>
       <c r="E29" s="49" t="s">
-        <v>188</v>
+        <v>176</v>
       </c>
       <c r="F29" s="49" t="s">
-        <v>190</v>
+        <v>178</v>
       </c>
       <c r="G29" s="49" t="s">
-        <v>191</v>
+        <v>179</v>
       </c>
       <c r="H29" s="49" t="s">
-        <v>181</v>
+        <v>169</v>
       </c>
       <c r="I29" s="49" t="s">
-        <v>192</v>
+        <v>180</v>
       </c>
       <c r="J29" s="49"/>
       <c r="K29" s="49">
         <v>0.64</v>
       </c>
       <c r="L29" s="49" t="s">
-        <v>193</v>
+        <v>181</v>
       </c>
       <c r="M29" s="50" t="s">
-        <v>194</v>
+        <v>182</v>
       </c>
       <c r="N29" s="51" t="s">
-        <v>50</v>
+        <v>45</v>
       </c>
     </row>
     <row r="32" spans="1:14" s="57" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A32" s="54" t="s">
-        <v>261</v>
+        <v>249</v>
       </c>
       <c r="B32" s="55" t="s">
-        <v>346</v>
+        <v>334</v>
       </c>
       <c r="C32" s="55"/>
       <c r="D32" s="55" t="s">
-        <v>274</v>
+        <v>262</v>
       </c>
       <c r="E32" s="55" t="s">
-        <v>275</v>
+        <v>263</v>
       </c>
       <c r="F32" s="55" t="s">
-        <v>276</v>
+        <v>264</v>
       </c>
       <c r="G32" s="55" t="s">
-        <v>279</v>
+        <v>267</v>
       </c>
       <c r="H32" s="55" t="s">
-        <v>280</v>
+        <v>268</v>
       </c>
       <c r="I32" s="55" t="s">
-        <v>280</v>
+        <v>268</v>
       </c>
       <c r="J32" s="55">
         <v>0.03</v>
       </c>
       <c r="K32" s="55" t="s">
-        <v>277</v>
+        <v>265</v>
       </c>
       <c r="L32" s="55" t="s">
-        <v>278</v>
-      </c>
-      <c r="M32" s="56"/>
+        <v>266</v>
+      </c>
+      <c r="M32" s="56" t="s">
+        <v>358</v>
+      </c>
     </row>
     <row r="33" spans="1:13" s="57" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A33" s="54" t="s">
-        <v>262</v>
+        <v>250</v>
       </c>
       <c r="B33" s="55" t="s">
-        <v>324</v>
+        <v>312</v>
       </c>
       <c r="C33" s="55" t="s">
-        <v>263</v>
+        <v>251</v>
       </c>
       <c r="D33" s="55" t="s">
-        <v>264</v>
+        <v>252</v>
       </c>
       <c r="E33" s="55" t="s">
-        <v>265</v>
+        <v>253</v>
       </c>
       <c r="F33" s="55" t="s">
-        <v>266</v>
+        <v>254</v>
       </c>
       <c r="G33" s="55" t="s">
-        <v>270</v>
+        <v>258</v>
       </c>
       <c r="H33" s="55" t="s">
-        <v>271</v>
+        <v>259</v>
       </c>
       <c r="I33" s="55" t="s">
-        <v>271</v>
+        <v>259</v>
       </c>
       <c r="J33" s="55">
         <v>0.3</v>
       </c>
       <c r="K33" s="55" t="s">
-        <v>267</v>
+        <v>255</v>
       </c>
       <c r="L33" s="55" t="s">
-        <v>268</v>
+        <v>256</v>
       </c>
       <c r="M33" s="56" t="s">
-        <v>269</v>
+        <v>257</v>
       </c>
     </row>
     <row r="37" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A37" s="12" t="s">
-        <v>305</v>
+        <v>293</v>
       </c>
       <c r="J37" s="9">
         <f>SUM(J3:J35)</f>
@@ -4890,13 +4901,13 @@
         <v>0</v>
       </c>
       <c r="B1" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="C1" s="8" t="s">
-        <v>11</v>
-      </c>
       <c r="D1" s="8" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
       <c r="E1" s="8" t="s">
         <v>1</v>
@@ -4905,16 +4916,16 @@
         <v>2</v>
       </c>
       <c r="G1" s="8" t="s">
-        <v>106</v>
+        <v>96</v>
       </c>
       <c r="H1" s="8" t="s">
         <v>3</v>
       </c>
       <c r="I1" s="8" t="s">
-        <v>107</v>
+        <v>97</v>
       </c>
       <c r="J1" s="8" t="s">
-        <v>94</v>
+        <v>89</v>
       </c>
       <c r="K1" s="8" t="s">
         <v>4</v>
@@ -4928,264 +4939,264 @@
     </row>
     <row r="3" spans="1:13" s="22" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
-        <v>281</v>
+        <v>269</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>347</v>
+        <v>335</v>
       </c>
       <c r="C3" s="2"/>
       <c r="D3" s="2" t="s">
-        <v>284</v>
+        <v>272</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>282</v>
+        <v>270</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>283</v>
+        <v>271</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>283</v>
+        <v>271</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>287</v>
+        <v>275</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>287</v>
+        <v>275</v>
       </c>
       <c r="J3" s="2">
         <v>0.31</v>
       </c>
       <c r="K3" s="2" t="s">
-        <v>286</v>
+        <v>274</v>
       </c>
       <c r="L3" s="2" t="s">
-        <v>285</v>
+        <v>273</v>
       </c>
       <c r="M3" s="21"/>
     </row>
     <row r="4" spans="1:13" s="22" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>325</v>
+        <v>313</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>61</v>
+        <v>56</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>211</v>
+        <v>199</v>
       </c>
       <c r="E4" s="31" t="s">
-        <v>204</v>
+        <v>192</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>206</v>
+        <v>194</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>207</v>
+        <v>195</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>203</v>
+        <v>191</v>
       </c>
       <c r="I4" s="2"/>
       <c r="J4" s="2">
         <v>0.1</v>
       </c>
       <c r="K4" s="2" t="s">
-        <v>208</v>
+        <v>196</v>
       </c>
       <c r="L4" s="2" t="s">
-        <v>209</v>
+        <v>197</v>
       </c>
       <c r="M4" s="21" t="s">
-        <v>296</v>
+        <v>284</v>
       </c>
     </row>
     <row r="5" spans="1:13" s="22" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>326</v>
+        <v>314</v>
       </c>
       <c r="C5" s="31" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>210</v>
+        <v>198</v>
       </c>
       <c r="E5" s="31" t="s">
-        <v>204</v>
+        <v>192</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>206</v>
+        <v>194</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>207</v>
+        <v>195</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>203</v>
+        <v>191</v>
       </c>
       <c r="I5" s="2"/>
       <c r="J5" s="2">
         <v>0.1</v>
       </c>
       <c r="K5" s="2" t="s">
-        <v>208</v>
+        <v>196</v>
       </c>
       <c r="L5" s="2" t="s">
-        <v>209</v>
+        <v>197</v>
       </c>
       <c r="M5" s="21"/>
     </row>
     <row r="6" spans="1:13" s="22" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>311</v>
+        <v>299</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>189</v>
+        <v>177</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>188</v>
+        <v>176</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>190</v>
+        <v>178</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>191</v>
+        <v>179</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>181</v>
+        <v>169</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>192</v>
+        <v>180</v>
       </c>
       <c r="I6" s="2"/>
       <c r="J6" s="2">
         <v>0.64</v>
       </c>
       <c r="K6" s="2" t="s">
-        <v>193</v>
+        <v>181</v>
       </c>
       <c r="L6" s="2" t="s">
-        <v>194</v>
+        <v>182</v>
       </c>
       <c r="M6" s="21" t="s">
-        <v>50</v>
+        <v>45</v>
       </c>
     </row>
     <row r="9" spans="1:13" s="24" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A9" s="3" t="s">
-        <v>288</v>
+        <v>276</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>348</v>
+        <v>336</v>
       </c>
       <c r="C9" s="4"/>
       <c r="D9" s="4" t="s">
-        <v>289</v>
+        <v>277</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>290</v>
+        <v>278</v>
       </c>
       <c r="F9" s="4" t="s">
-        <v>291</v>
+        <v>279</v>
       </c>
       <c r="G9" s="4" t="s">
-        <v>294</v>
+        <v>282</v>
       </c>
       <c r="H9" s="4" t="s">
-        <v>295</v>
+        <v>283</v>
       </c>
       <c r="I9" s="4" t="s">
-        <v>295</v>
+        <v>283</v>
       </c>
       <c r="J9" s="4">
         <v>0.48</v>
       </c>
       <c r="K9" s="4" t="s">
-        <v>293</v>
+        <v>281</v>
       </c>
       <c r="L9" s="4" t="s">
-        <v>292</v>
+        <v>280</v>
       </c>
       <c r="M9" s="23"/>
     </row>
     <row r="12" spans="1:13" s="26" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A12" s="6" t="s">
-        <v>304</v>
+        <v>292</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>349</v>
+        <v>337</v>
       </c>
       <c r="C12" s="7"/>
       <c r="D12" s="7" t="s">
-        <v>284</v>
+        <v>272</v>
       </c>
       <c r="E12" s="7" t="s">
-        <v>282</v>
+        <v>270</v>
       </c>
       <c r="F12" s="7" t="s">
-        <v>283</v>
+        <v>271</v>
       </c>
       <c r="G12" s="7" t="s">
-        <v>283</v>
+        <v>271</v>
       </c>
       <c r="H12" s="7" t="s">
-        <v>287</v>
+        <v>275</v>
       </c>
       <c r="I12" s="7" t="s">
-        <v>287</v>
+        <v>275</v>
       </c>
       <c r="J12" s="7">
         <v>0.31</v>
       </c>
       <c r="K12" s="7" t="s">
-        <v>286</v>
+        <v>274</v>
       </c>
       <c r="L12" s="7" t="s">
-        <v>285</v>
+        <v>273</v>
       </c>
       <c r="M12" s="25"/>
     </row>
     <row r="13" spans="1:13" s="26" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A13" s="6" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>327</v>
+        <v>315</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="D13" s="7" t="s">
-        <v>210</v>
+        <v>198</v>
       </c>
       <c r="E13" s="34" t="s">
-        <v>204</v>
+        <v>192</v>
       </c>
       <c r="F13" s="7" t="s">
-        <v>206</v>
+        <v>194</v>
       </c>
       <c r="G13" s="7" t="s">
-        <v>207</v>
+        <v>195</v>
       </c>
       <c r="H13" s="7" t="s">
-        <v>203</v>
+        <v>191</v>
       </c>
       <c r="I13" s="7"/>
       <c r="J13" s="7">
         <v>0.1</v>
       </c>
       <c r="K13" s="7" t="s">
-        <v>208</v>
+        <v>196</v>
       </c>
       <c r="L13" s="7" t="s">
-        <v>209</v>
+        <v>197</v>
       </c>
       <c r="M13" s="25"/>
     </row>
@@ -5197,81 +5208,81 @@
     </row>
     <row r="16" spans="1:13" s="29" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A16" s="16" t="s">
-        <v>303</v>
+        <v>291</v>
       </c>
       <c r="B16" s="10" t="s">
-        <v>350</v>
+        <v>338</v>
       </c>
       <c r="C16" s="10"/>
       <c r="D16" s="10" t="s">
-        <v>284</v>
+        <v>272</v>
       </c>
       <c r="E16" s="10" t="s">
-        <v>282</v>
+        <v>270</v>
       </c>
       <c r="F16" s="10" t="s">
-        <v>283</v>
+        <v>271</v>
       </c>
       <c r="G16" s="10" t="s">
-        <v>283</v>
+        <v>271</v>
       </c>
       <c r="H16" s="10" t="s">
-        <v>287</v>
+        <v>275</v>
       </c>
       <c r="I16" s="10" t="s">
-        <v>287</v>
+        <v>275</v>
       </c>
       <c r="J16" s="10">
         <v>0.31</v>
       </c>
       <c r="K16" s="10" t="s">
-        <v>286</v>
+        <v>274</v>
       </c>
       <c r="L16" s="10" t="s">
-        <v>285</v>
+        <v>273</v>
       </c>
       <c r="M16" s="28"/>
     </row>
     <row r="17" spans="1:13" s="29" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A17" s="16" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="B17" s="10" t="s">
-        <v>328</v>
+        <v>316</v>
       </c>
       <c r="C17" s="10" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="D17" s="10" t="s">
-        <v>210</v>
+        <v>198</v>
       </c>
       <c r="E17" s="27" t="s">
-        <v>204</v>
+        <v>192</v>
       </c>
       <c r="F17" s="10" t="s">
-        <v>206</v>
+        <v>194</v>
       </c>
       <c r="G17" s="10" t="s">
-        <v>207</v>
+        <v>195</v>
       </c>
       <c r="H17" s="10" t="s">
-        <v>203</v>
+        <v>191</v>
       </c>
       <c r="I17" s="10"/>
       <c r="J17" s="10">
         <v>0.1</v>
       </c>
       <c r="K17" s="10" t="s">
-        <v>208</v>
+        <v>196</v>
       </c>
       <c r="L17" s="10" t="s">
-        <v>209</v>
+        <v>197</v>
       </c>
       <c r="M17" s="28"/>
     </row>
     <row r="21" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A21" s="12" t="s">
-        <v>305</v>
+        <v>293</v>
       </c>
       <c r="J21" s="9">
         <f>SUM(J3:J17)</f>

</xml_diff>